<commit_message>
Añadir hoja masiva (bulksheet) para crear 'Pinza - Principal V2' y 'Pinza - Pruebas'
Rellena la plantilla oficial de Juan: 2 campañas nuevas en pausa, grupos,
anuncio, 10 keywords, 8 negativas, 4 ASIN de competencia y la propia
ficha como producto negativo. El Excel de seguimiento pasa a usar la
campaña nueva.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8zFsXd31MYxmY7hRPcJU8
</commit_message>
<xml_diff>
--- a/resultados/grupo_pinza_V2.xlsx
+++ b/resultados/grupo_pinza_V2.xlsx
@@ -38,7 +38,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Es la campaña donde la pinza ha vendido (grupo 'Pinza', 99% del gasto de la pinza). Su grupo antiguo 'Pinza' tiene estas mismas keywords: debe seguir EN PAUSA para no pujar contra ti mismo. Alternativa: campaña nueva solo para este grupo (control de presupuesto más limpio).</t>
+          <t xml:space="preserve">Campaña nueva (presupuesto propio de ~1,67 €/día). La antigua 'Soporte móvil pinza' (ID A0335903WCRWL9CYXAOF) tiene estas mismas keywords en su grupo 'Pinza': debe seguir EN PAUSA para no pujar contra ti mismo.</t>
         </r>
       </text>
     </comment>
@@ -315,7 +315,7 @@
     <t xml:space="preserve">Campaña</t>
   </si>
   <si>
-    <t xml:space="preserve">Soporte móvil pinza  (ID A0335903WCRWL9CYXAOF)</t>
+    <t xml:space="preserve">Pinza - Principal V2 (NUEVA, se crea con resultados/hoja_masiva_pinza_V2.xlsx)</t>
   </si>
   <si>
     <t xml:space="preserve">Tipo de campaña</t>
@@ -726,7 +726,7 @@
     <t xml:space="preserve">Crear grupo de anuncios</t>
   </si>
   <si>
-    <t xml:space="preserve">Crear 'Pinza - Principal V2' con el anuncio B0DCZS1NR6 (O8-5W7J-DSK1) y las 10 keywords de T-002…T-011. Objetivo: concentrar el gasto en lo que ya vende y en 5 frases nuevas con alta intención, con ACOS ≤ 35%.</t>
+    <t xml:space="preserve">Crear la campaña y el grupo 'Pinza - Principal V2' (hoja masiva) con el anuncio B0DCZS1NR6 (O8-5W7J-DSK1) y las 10 keywords de T-002…T-011. Objetivo: concentrar el gasto en lo que ya vende y en 5 frases nuevas con alta intención, con ACOS ≤ 35%.</t>
   </si>
   <si>
     <t xml:space="preserve">Pendiente de aplicar</t>

</xml_diff>